<commit_message>
Add sample-wise median regression fits for pressure and temperature results
</commit_message>
<xml_diff>
--- a/input.xlsx
+++ b/input.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\13493\Documents\PROJECTS\Cpx_thermobarometry_recommend_202507\code\AIMS4PT\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{08519F5D-D717-402B-B33E-193FB0344BEE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2E8BCA50-7AEB-4A00-AD85-864BB9242422}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="4020" yWindow="1860" windowWidth="19200" windowHeight="11170" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="compositions" sheetId="1" r:id="rId1"/>
@@ -407,6 +407,7 @@
     <xf numFmtId="0" fontId="9" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="8" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -425,7 +426,6 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="8" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -441,10 +441,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -739,32 +735,32 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:23" x14ac:dyDescent="0.35">
-      <c r="B1" s="9" t="s">
+      <c r="B1" s="10" t="s">
         <v>23</v>
       </c>
-      <c r="C1" s="10"/>
-      <c r="D1" s="10"/>
-      <c r="E1" s="10"/>
-      <c r="F1" s="10"/>
-      <c r="G1" s="10"/>
-      <c r="H1" s="10"/>
-      <c r="I1" s="10"/>
-      <c r="J1" s="10"/>
-      <c r="K1" s="11"/>
-      <c r="L1" s="12" t="s">
+      <c r="C1" s="11"/>
+      <c r="D1" s="11"/>
+      <c r="E1" s="11"/>
+      <c r="F1" s="11"/>
+      <c r="G1" s="11"/>
+      <c r="H1" s="11"/>
+      <c r="I1" s="11"/>
+      <c r="J1" s="11"/>
+      <c r="K1" s="12"/>
+      <c r="L1" s="13" t="s">
         <v>29</v>
       </c>
-      <c r="M1" s="13"/>
-      <c r="N1" s="13"/>
-      <c r="O1" s="13"/>
-      <c r="P1" s="13"/>
-      <c r="Q1" s="13"/>
-      <c r="R1" s="13"/>
-      <c r="S1" s="13"/>
-      <c r="T1" s="13"/>
-      <c r="U1" s="13"/>
-      <c r="V1" s="13"/>
-      <c r="W1" s="14"/>
+      <c r="M1" s="14"/>
+      <c r="N1" s="14"/>
+      <c r="O1" s="14"/>
+      <c r="P1" s="14"/>
+      <c r="Q1" s="14"/>
+      <c r="R1" s="14"/>
+      <c r="S1" s="14"/>
+      <c r="T1" s="14"/>
+      <c r="U1" s="14"/>
+      <c r="V1" s="14"/>
+      <c r="W1" s="15"/>
     </row>
     <row r="2" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A2" s="2" t="s">
@@ -899,7 +895,7 @@
       <c r="V3">
         <v>0.27</v>
       </c>
-      <c r="W3" s="15">
+      <c r="W3" s="9">
         <v>0</v>
       </c>
     </row>
@@ -965,7 +961,7 @@
       <c r="V4">
         <v>0.34</v>
       </c>
-      <c r="W4" s="15">
+      <c r="W4" s="9">
         <v>0</v>
       </c>
     </row>
@@ -1031,7 +1027,7 @@
       <c r="V5">
         <v>0.4</v>
       </c>
-      <c r="W5" s="15">
+      <c r="W5" s="9">
         <v>0</v>
       </c>
     </row>
@@ -1097,7 +1093,7 @@
       <c r="V6">
         <v>0.13</v>
       </c>
-      <c r="W6" s="15">
+      <c r="W6" s="9">
         <v>0</v>
       </c>
     </row>
@@ -1163,7 +1159,7 @@
       <c r="V7">
         <v>0.16</v>
       </c>
-      <c r="W7" s="15">
+      <c r="W7" s="9">
         <v>0</v>
       </c>
     </row>
@@ -1178,7 +1174,7 @@
       <c r="I8" s="6"/>
       <c r="J8" s="6"/>
       <c r="K8" s="7"/>
-      <c r="W8" s="15"/>
+      <c r="W8" s="9"/>
     </row>
     <row r="9" spans="1:23" x14ac:dyDescent="0.35">
       <c r="B9" s="5"/>
@@ -1191,7 +1187,7 @@
       <c r="I9" s="6"/>
       <c r="J9" s="6"/>
       <c r="K9" s="7"/>
-      <c r="W9" s="15"/>
+      <c r="W9" s="9"/>
     </row>
     <row r="10" spans="1:23" x14ac:dyDescent="0.35">
       <c r="B10" s="5"/>
@@ -1204,7 +1200,7 @@
       <c r="I10" s="6"/>
       <c r="J10" s="6"/>
       <c r="K10" s="7"/>
-      <c r="W10" s="15"/>
+      <c r="W10" s="9"/>
     </row>
     <row r="11" spans="1:23" x14ac:dyDescent="0.35">
       <c r="B11" s="5"/>
@@ -1217,7 +1213,7 @@
       <c r="I11" s="6"/>
       <c r="J11" s="6"/>
       <c r="K11" s="7"/>
-      <c r="W11" s="15"/>
+      <c r="W11" s="9"/>
     </row>
     <row r="12" spans="1:23" x14ac:dyDescent="0.35">
       <c r="B12" s="5"/>
@@ -1230,7 +1226,7 @@
       <c r="I12" s="6"/>
       <c r="J12" s="6"/>
       <c r="K12" s="7"/>
-      <c r="W12" s="15"/>
+      <c r="W12" s="9"/>
     </row>
     <row r="13" spans="1:23" x14ac:dyDescent="0.35">
       <c r="B13" s="5"/>
@@ -1243,7 +1239,7 @@
       <c r="I13" s="6"/>
       <c r="J13" s="6"/>
       <c r="K13" s="7"/>
-      <c r="W13" s="15"/>
+      <c r="W13" s="9"/>
     </row>
     <row r="14" spans="1:23" x14ac:dyDescent="0.35">
       <c r="B14" s="5"/>
@@ -1256,7 +1252,7 @@
       <c r="I14" s="6"/>
       <c r="J14" s="6"/>
       <c r="K14" s="7"/>
-      <c r="W14" s="15"/>
+      <c r="W14" s="9"/>
     </row>
     <row r="15" spans="1:23" x14ac:dyDescent="0.35">
       <c r="B15" s="5"/>
@@ -1270,7 +1266,7 @@
       <c r="J15" s="6"/>
       <c r="K15" s="7"/>
       <c r="P15" s="4"/>
-      <c r="W15" s="15"/>
+      <c r="W15" s="9"/>
     </row>
     <row r="16" spans="1:23" x14ac:dyDescent="0.35">
       <c r="W16" s="3"/>

</xml_diff>